<commit_message>
feat: redesign calculator for client meetings with light UI, Yandex mailboxes counter and conclusions
</commit_message>
<xml_diff>
--- a/КАЛЬКУЛЯТОР_ОКУПАЕМОСТИ_CALLTALK.xlsx
+++ b/КАЛЬКУЛЯТОР_ОКУПАЕМОСТИ_CALLTALK.xlsx
@@ -17,14 +17,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="+0%"/>
     <numFmt numFmtId="166" formatCode="0.0x"/>
-    <numFmt numFmtId="167" formatCode="0 &quot;сделок&quot;"/>
-    <numFmt numFmtId="168" formatCode="#,##0 руб."/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -98,17 +96,11 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <i val="1"/>
       <color rgb="001E1B4B"/>
       <sz val="10"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="00475569"/>
-      <sz val="9"/>
-    </font>
   </fonts>
-  <fills count="11">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -163,12 +155,6 @@
         <bgColor rgb="0014152A"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F8FAFC"/>
-        <bgColor rgb="00F8FAFC"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -210,7 +196,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -240,7 +226,6 @@
     <xf numFmtId="3" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -269,11 +254,6 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -644,43 +624,43 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
     <col width="4" customWidth="1" min="4" max="4"/>
     <col width="32" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ЭКСПРЕСС-КАЛЬКУЛЯТОР ОКУПАЕМОСТИ CALL-TALK</t>
+          <t>КАЛЬКУЛЯТОР ОКУПАЕМОСТИ B2B-АУТРИЧА CALL-TALK</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Жёлтые ячейки заполняем вручную со слов клиента. Главное по окупаемости — сразу наверху в правом блоке! Второстепенное — сдвинуто ниже.</t>
+          <t>Жёлтые ячейки заполняются со слов клиента на встрече. Точка безубыточности и выводы — сразу наверху в правом блоке.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>1. ЧТО ВВОДИТ МЕНЕДЖЕР (РУЧНОЙ ВВОД)</t>
+          <t>1. ПАРАМЕТРЫ ПРОЕКТА (ВВОД ДАННЫХ)</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>2. ГЛАВНОЕ: ОКУПАЕМОСТЬ И ТОЧКА БЕЗУБЫТОЧНОСТИ (САМЫЙ ВЕРХ)</t>
+          <t>2. ГЛАВНОЕ: ОКУПАЕМОСТЬ И ТОЧКА БЕЗУБЫТОЧНОСТИ</t>
         </is>
       </c>
     </row>
@@ -695,7 +675,7 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>2, 3 или 4. Основной срок — 4</t>
+          <t>2 или 4 мес. Основной срок — 4</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
@@ -753,11 +733,11 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>НУЖНАЯ КОНВЕРСИЯ В СДЕЛКУ:</t>
+          <t>НЕОБХОДИМАЯ КОНВЕРСИЯ В СДЕЛКУ:</t>
         </is>
       </c>
       <c r="F6" s="15">
-        <f>F4/B12</f>
+        <f>F4/B11</f>
         <v/>
       </c>
       <c r="G6" s="8" t="inlineStr">
@@ -786,24 +766,22 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Оценка клиента, дефолт 15% (или 10%)</t>
+          <t>Оценка отдела продаж клиента (дефолт 15%)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Уровень цены лида</t>
-        </is>
-      </c>
-      <c r="B8" s="17" t="inlineStr">
-        <is>
-          <t>Уровень 2</t>
-        </is>
+          <t>Почтовые ящики Яндекс 360, шт.</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>10</v>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Выберите: Уровень 1, Уровень 2 или Уровень 3</t>
+          <t>10 (база), 20 (масштаб) или 30 ящиков</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
@@ -811,8 +789,8 @@
           <t>Прогноз закрытых сделок, шт.:</t>
         </is>
       </c>
-      <c r="F8" s="18">
-        <f>ROUND(B12*B7, 0)</f>
+      <c r="F8" s="17">
+        <f>ROUND(B11*B7, 0)</f>
         <v/>
       </c>
       <c r="G8" s="8" t="inlineStr">
@@ -833,29 +811,31 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Своя цена лида, руб.</t>
-        </is>
-      </c>
-      <c r="B9" s="13" t="inlineStr"/>
+          <t>Ставка за 1 лид, руб.</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="n">
+        <v>2800</v>
+      </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Пусто = цена уровня (если согласована своя)</t>
+          <t>Оплата за лид с подтвержденным интересом</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Итоговая ставка за лид, руб.</t>
-        </is>
-      </c>
-      <c r="B10" s="19">
-        <f>IF(B9&lt;&gt;"",B9,INDEX('Справочник'!$B$13:$B$15,MATCH(B8,'Справочник'!$A$13:$A$15,0)))</f>
+          <t>Фикс в месяц, руб.</t>
+        </is>
+      </c>
+      <c r="B10" s="18">
+        <f>INDEX('Справочник'!$B$6:$B$8,MATCH(B4,'Справочник'!$A$6:$A$8,0))</f>
         <v/>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Ставка за 1 лид с интересом</t>
+          <t>Из справочника по сроку договора</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
@@ -863,8 +843,8 @@
           <t>ОБЩИЙ БЮДЖЕТ CALL-TALK, руб.:</t>
         </is>
       </c>
-      <c r="F10" s="20">
-        <f>B11*B4+B12*B10</f>
+      <c r="F10" s="19">
+        <f>B10*B4+B11*B9</f>
         <v/>
       </c>
       <c r="G10" s="8" t="inlineStr">
@@ -872,7 +852,7 @@
           <t>ОКУПАЕМОСТЬ ЗАТРАТ (ROI), %:</t>
         </is>
       </c>
-      <c r="H10" s="21">
+      <c r="H10" s="20">
         <f>H6/F10</f>
         <v/>
       </c>
@@ -885,56 +865,56 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Фикс в месяц, руб.</t>
-        </is>
-      </c>
-      <c r="B11" s="19">
-        <f>INDEX('Справочник'!$B$6:$B$8,MATCH(B4,'Справочник'!$A$6:$A$8,0))</f>
+          <t>Прогноз лидов за срок, шт.</t>
+        </is>
+      </c>
+      <c r="B11" s="6">
+        <f>IF(B4=4,78,IF(B4=2,34,56))</f>
         <v/>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Из справочника по сроку договора</t>
+          <t>Дефолт тарифа (4 мес: 78, 2 мес: 34) или вручную</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Прогноз лидов за срок, шт.</t>
-        </is>
-      </c>
-      <c r="B12" s="6">
-        <f>IF(B4=4,78,IF(B4=2,34,56))</f>
+          <t>Затраты на Яндекс 360 (~300 руб./ящик в мес), руб.</t>
+        </is>
+      </c>
+      <c r="B12" s="18">
+        <f>B8*B4*300</f>
         <v/>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Дефолт тарифа (4 мес: 78, 2 мес: 34) или вручную</t>
-        </is>
-      </c>
-      <c r="E12" s="22" t="inlineStr">
-        <is>
-          <t>ЧТО СКАЗАТЬ КЛИЕНТУ НА ВСТРЕЧЕ (ГОТОВЫЙ РЕЧЕВОЙ МОДУЛЬ):</t>
+          <t>Оплачивает клиент Яндексу или нам под ключ</t>
+        </is>
+      </c>
+      <c r="E12" s="21" t="inlineStr">
+        <is>
+          <t>ВЫВОДЫ ПО ОКУПАЕМОСТИ ДЛЯ КЛИЕНТА:</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="E13" s="23">
-        <f>"«За "&amp;B4&amp;" мес. мы передадим вам "&amp;B12&amp;" лидов с интересом. Ваши суммарные инвестиции — "&amp;TEXT(F10,"#,##0")&amp;" руб. При среднем чеке "&amp;TEXT(B5,"#,##0")&amp;" руб. и чистой марже "&amp;TEXT(B6,"0%")&amp;" валовая прибыль со сделки составляет "&amp;TEXT(H4,"#,##0")&amp;" руб. "&amp;"Поэтому для полной окупаемости вам достаточно закрыть всего "&amp;F4&amp;" из "&amp;B12&amp;" лидов "&amp;"(конверсия всего "&amp;TEXT(F6,"0.0%")&amp;"). Всё, что вы закроете сверх этого (еще "&amp;(F8-F4)&amp;" сделок на чистую прибыль "&amp;TEXT((F8-F4)*H4,"#,##0")&amp;" руб.), остаётся вашей чистой прибылью сверх затрат на запуск!»"</f>
+      <c r="E13" s="22">
+        <f>"1. Для 100% возврата бюджета ("&amp;TEXT(F10,"#,##0")&amp;" руб.) достаточно закрыть ВСЕГО "&amp;F4&amp;" сделок из "&amp;B11&amp;" лидов (конверсия всего "&amp;TEXT(F6,"0.0%")&amp;")."&amp;CHAR(10)&amp;"2. Финансовый результат: при конверсии "&amp;TEXT(B7,"0%")&amp;" закрывается "&amp;F8&amp;" сделок на "&amp;TEXT(F8*B5,"#,##0")&amp;" руб. выручки и +"&amp;TEXT(H6,"#,##0")&amp;" руб. чистой прибыли (ROI "&amp;TEXT(H10,"+0%")&amp;")."&amp;CHAR(10)&amp;"3. Инфраструктура: "&amp;B8&amp;" ящиков Яндекс 360. Оплата лидов строго за подтвержденный интерес. Нецелевые ответы — 0 руб."</f>
         <v/>
       </c>
     </row>
     <row r="14"/>
     <row r="16">
-      <c r="A16" s="24" t="inlineStr">
+      <c r="A16" s="23" t="inlineStr">
         <is>
           <t>3. ВТОРОСТЕПЕННЫЕ ПОКАЗАТЕЛИ И ДЕТАЛИЗАЦИЯ (СДВИНУТЫ НИЖЕ)</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="E17" s="25" t="inlineStr">
+      <c r="E17" s="24" t="inlineStr">
         <is>
           <t>ПОМЕСЯЧНАЯ ВОРОНКА И ГРАФИК ПЛАТЕЖЕЙ</t>
         </is>
@@ -946,7 +926,7 @@
           <t>Привлеченный оборот (выручка), руб.</t>
         </is>
       </c>
-      <c r="B18" s="26">
+      <c r="B18" s="25">
         <f>F8*B5</f>
         <v/>
       </c>
@@ -955,27 +935,27 @@
           <t>Сделки × Чек</t>
         </is>
       </c>
-      <c r="E18" s="27" t="inlineStr">
+      <c r="E18" s="26" t="inlineStr">
         <is>
           <t>Месяц</t>
         </is>
       </c>
-      <c r="F18" s="27" t="inlineStr">
+      <c r="F18" s="26" t="inlineStr">
         <is>
           <t>Лидов, шт.</t>
         </is>
       </c>
-      <c r="G18" s="27" t="inlineStr">
+      <c r="G18" s="26" t="inlineStr">
         <is>
           <t>Лиды, руб.</t>
         </is>
       </c>
-      <c r="H18" s="27" t="inlineStr">
+      <c r="H18" s="26" t="inlineStr">
         <is>
           <t>Фикс, руб.</t>
         </is>
       </c>
-      <c r="I18" s="27" t="inlineStr">
+      <c r="I18" s="26" t="inlineStr">
         <is>
           <t>Итого за месяц, руб.</t>
         </is>
@@ -987,7 +967,7 @@
           <t>Доля расходов Call-Talk в обороте, %</t>
         </is>
       </c>
-      <c r="B19" s="28">
+      <c r="B19" s="27">
         <f>F10/B18</f>
         <v/>
       </c>
@@ -1004,15 +984,15 @@
       <c r="F19" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="G19" s="29">
-        <f>F19*$B$10</f>
-        <v/>
-      </c>
-      <c r="H19" s="29">
-        <f>IF(1&lt;=$B$4,$B$11,0)</f>
-        <v/>
-      </c>
-      <c r="I19" s="29">
+      <c r="G19" s="28">
+        <f>F19*$B$9</f>
+        <v/>
+      </c>
+      <c r="H19" s="28">
+        <f>IF(1&lt;=$B$4,$B$10,0)</f>
+        <v/>
+      </c>
+      <c r="I19" s="28">
         <f>G19+H19</f>
         <v/>
       </c>
@@ -1023,7 +1003,7 @@
           <t>Стоимость привлечения клиента (CAC), руб.</t>
         </is>
       </c>
-      <c r="B20" s="26">
+      <c r="B20" s="25">
         <f>F10/F8</f>
         <v/>
       </c>
@@ -1038,18 +1018,18 @@
         </is>
       </c>
       <c r="F20" s="5">
-        <f>ROUND(($B$12-11)/($B$4-1), 0)</f>
-        <v/>
-      </c>
-      <c r="G20" s="29">
-        <f>F20*$B$10</f>
-        <v/>
-      </c>
-      <c r="H20" s="29">
-        <f>IF(2&lt;=$B$4,$B$11,0)</f>
-        <v/>
-      </c>
-      <c r="I20" s="29">
+        <f>ROUND(($B$11-11)/($B$4-1), 0)</f>
+        <v/>
+      </c>
+      <c r="G20" s="28">
+        <f>F20*$B$9</f>
+        <v/>
+      </c>
+      <c r="H20" s="28">
+        <f>IF(2&lt;=$B$4,$B$10,0)</f>
+        <v/>
+      </c>
+      <c r="I20" s="28">
         <f>G20+H20</f>
         <v/>
       </c>
@@ -1060,8 +1040,8 @@
           <t>Платеж при старте (фикс за весь срок), руб.</t>
         </is>
       </c>
-      <c r="B21" s="26">
-        <f>B11*B4</f>
+      <c r="B21" s="25">
+        <f>B10*B4</f>
         <v/>
       </c>
       <c r="C21" s="7" t="inlineStr">
@@ -1075,18 +1055,18 @@
         </is>
       </c>
       <c r="F21" s="5">
-        <f>IF(3&lt;=$B$4,ROUND(($B$12-11)/($B$4-1), 0),0)</f>
-        <v/>
-      </c>
-      <c r="G21" s="29">
-        <f>F21*$B$10</f>
-        <v/>
-      </c>
-      <c r="H21" s="29">
-        <f>IF(3&lt;=$B$4,$B$11,0)</f>
-        <v/>
-      </c>
-      <c r="I21" s="29">
+        <f>IF(3&lt;=$B$4,ROUND(($B$11-11)/($B$4-1), 0),0)</f>
+        <v/>
+      </c>
+      <c r="G21" s="28">
+        <f>F21*$B$9</f>
+        <v/>
+      </c>
+      <c r="H21" s="28">
+        <f>IF(3&lt;=$B$4,$B$10,0)</f>
+        <v/>
+      </c>
+      <c r="I21" s="28">
         <f>G21+H21</f>
         <v/>
       </c>
@@ -1097,7 +1077,7 @@
           <t>Кратность возврата бюджета (ROMI), раз</t>
         </is>
       </c>
-      <c r="B22" s="30">
+      <c r="B22" s="29">
         <f>H8/F10</f>
         <v/>
       </c>
@@ -1112,145 +1092,51 @@
         </is>
       </c>
       <c r="F22" s="5">
-        <f>IF(4&lt;=$B$4,$B$12-11-F20-F21,0)</f>
-        <v/>
-      </c>
-      <c r="G22" s="29">
-        <f>F22*$B$10</f>
-        <v/>
-      </c>
-      <c r="H22" s="29">
-        <f>IF(4&lt;=$B$4,$B$11,0)</f>
-        <v/>
-      </c>
-      <c r="I22" s="29">
+        <f>IF(4&lt;=$B$4,$B$11-11-F20-F21,0)</f>
+        <v/>
+      </c>
+      <c r="G22" s="28">
+        <f>F22*$B$9</f>
+        <v/>
+      </c>
+      <c r="H22" s="28">
+        <f>IF(4&lt;=$B$4,$B$10,0)</f>
+        <v/>
+      </c>
+      <c r="I22" s="28">
         <f>G22+H22</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="E23" s="31" t="inlineStr">
+      <c r="E23" s="30" t="inlineStr">
         <is>
           <t>ИТОГО</t>
         </is>
       </c>
-      <c r="F23" s="31">
+      <c r="F23" s="30">
         <f>SUM(F19:F22)</f>
         <v/>
       </c>
-      <c r="G23" s="19">
+      <c r="G23" s="18">
         <f>SUM(G19:G22)</f>
         <v/>
       </c>
-      <c r="H23" s="19">
+      <c r="H23" s="18">
         <f>SUM(H19:H22)</f>
         <v/>
       </c>
-      <c r="I23" s="19">
+      <c r="I23" s="18">
         <f>SUM(I19:I22)</f>
         <v/>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="22" t="inlineStr">
-        <is>
-          <t>ТАБЛИЦА: ОКУПАЕМОСТЬ ПРИ РАЗНОЙ МАРЖЕ</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>Маржа 8% (супер-консервативно)</t>
-        </is>
-      </c>
-      <c r="B25" s="32">
-        <f>ROUNDUP($F$10/($B$5*0.08), 0)</f>
-        <v/>
-      </c>
-      <c r="C25" s="33">
-        <f>($F$8*$B$5*0.08)-$F$10</f>
-        <v/>
-      </c>
-      <c r="E25" s="34" t="inlineStr">
-        <is>
-          <t>ПАМЯТКА ДЛЯ МЕНЕДЖЕРА CALL-TALK:
-• Стандарт маржи Call-Talk: всегда закладываем маржу 10–12% (максимум 15%), чтобы не завышать окупаемость.
-• Не перегружайте клиента: начинайте диалог с Точки безубыточности («Вам достаточно закрыть всего 2–3 сделки из 78!»).
-• Фикс за инфраструктуру оплачивается единоразово на старте за весь срок договора.
-• Лиды оплачиваются помесячно по факту подтвержденного интереса. Отказы и спам — 0 руб..
-• Договорное исключение: если ЛПР не ответил после 3 попыток за 5 дней — лид списывается в 0 руб..</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="12" t="inlineStr">
-        <is>
-          <t>Маржа 10% (консервативно)</t>
-        </is>
-      </c>
-      <c r="B26" s="32">
-        <f>ROUNDUP($F$10/($B$5*0.1), 0)</f>
-        <v/>
-      </c>
-      <c r="C26" s="33">
-        <f>($F$8*$B$5*0.1)-$F$10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="12" t="inlineStr">
-        <is>
-          <t>Маржа 12% (стандарт B2B)</t>
-        </is>
-      </c>
-      <c r="B27" s="32">
-        <f>ROUNDUP($F$10/($B$5*0.12), 0)</f>
-        <v/>
-      </c>
-      <c r="C27" s="33">
-        <f>($F$8*$B$5*0.12)-$F$10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="12" t="inlineStr">
-        <is>
-          <t>Маржа 15% (максимальный ориентир)</t>
-        </is>
-      </c>
-      <c r="B28" s="32">
-        <f>ROUNDUP($F$10/($B$5*0.15), 0)</f>
-        <v/>
-      </c>
-      <c r="C28" s="33">
-        <f>($F$8*$B$5*0.15)-$F$10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t>Маржа 20% (только для сервиса/IT)</t>
-        </is>
-      </c>
-      <c r="B29" s="32">
-        <f>ROUNDUP($F$10/($B$5*0.2), 0)</f>
-        <v/>
-      </c>
-      <c r="C29" s="33">
-        <f>($F$8*$B$5*0.2)-$F$10</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="6">
     <mergeCell ref="E3:I3"/>
     <mergeCell ref="E13:I14"/>
     <mergeCell ref="E12:I12"/>
-    <mergeCell ref="E25:I29"/>
     <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A24:C24"/>
     <mergeCell ref="E17:I17"/>
     <mergeCell ref="A16:I16"/>
   </mergeCells>
@@ -1264,12 +1150,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="45" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -1290,7 +1176,7 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>ФИКС ПО СРОКАМ</t>
+          <t>ФИКС ПО СРОКАМ ДОГОВОРА</t>
         </is>
       </c>
     </row>
@@ -1317,122 +1203,53 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="35" t="n">
+      <c r="A6" s="31" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="36" t="n">
+      <c r="B6" s="32" t="n">
         <v>56000</v>
       </c>
-      <c r="C6" s="36">
+      <c r="C6" s="32">
         <f>A6*B6</f>
         <v/>
       </c>
-      <c r="D6" s="37" t="inlineStr">
+      <c r="D6" s="33" t="inlineStr">
         <is>
           <t>Тестовый пилот (по согласованию)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="35" t="n">
+      <c r="A7" s="31" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="36" t="n">
+      <c r="B7" s="32" t="n">
         <v>48000</v>
       </c>
-      <c r="C7" s="36">
+      <c r="C7" s="32">
         <f>A7*B7</f>
         <v/>
       </c>
-      <c r="D7" s="37" t="inlineStr">
+      <c r="D7" s="33" t="inlineStr">
         <is>
           <t>Промежуточный тариф</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="35" t="n">
+      <c r="A8" s="31" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="36" t="n">
+      <c r="B8" s="32" t="n">
         <v>39000</v>
       </c>
-      <c r="C8" s="36">
+      <c r="C8" s="32">
         <f>A8*B8</f>
         <v/>
       </c>
-      <c r="D8" s="37" t="inlineStr">
+      <c r="D8" s="33" t="inlineStr">
         <is>
           <t>Основной флагманский срок (скидка 46%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>УРОВНИ ЦЕНЫ ЛИДА (по профилю целевой аудитории покупателей)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Уровень</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Цена лида, руб.</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Профиль целевой аудитории покупателей</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="35" t="inlineStr">
-        <is>
-          <t>Уровень 1</t>
-        </is>
-      </c>
-      <c r="B13" s="36" t="n">
-        <v>1800</v>
-      </c>
-      <c r="C13" s="37" t="inlineStr">
-        <is>
-          <t>Малый бизнес / ИП: выручка ЦА до 500 млн руб., штат до 100 чел., чек до 500 тыс. руб.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="35" t="inlineStr">
-        <is>
-          <t>Уровень 2</t>
-        </is>
-      </c>
-      <c r="B14" s="36" t="n">
-        <v>2800</v>
-      </c>
-      <c r="C14" s="37" t="inlineStr">
-        <is>
-          <t>Средний бизнес (Дефолт): выручка 500 млн – 1,5 млрд руб., штат 100–250 чел., чек 0,5–3 млн руб.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="35" t="inlineStr">
-        <is>
-          <t>Уровень 3</t>
-        </is>
-      </c>
-      <c r="B15" s="36" t="n">
-        <v>4800</v>
-      </c>
-      <c r="C15" s="37" t="inlineStr">
-        <is>
-          <t>Крупный бизнес / Enterprise: выручка от 1,5 млрд руб., C-level ЛПР, чек от 3 млн руб.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add 15 mailboxes, 30k/50k/100k check pills, 20/25/30/50% margin pills, 30% conv pill, and LTV pills
</commit_message>
<xml_diff>
--- a/КАЛЬКУЛЯТОР_ОКУПАЕМОСТИ_CALLTALK.xlsx
+++ b/КАЛЬКУЛЯТОР_ОКУПАЕМОСТИ_CALLTALK.xlsx
@@ -781,7 +781,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>10 (база), 20 (масштаб) или 30 ящиков</t>
+          <t>10, 15, 20 или 30 ящиков</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
@@ -869,12 +869,12 @@
         </is>
       </c>
       <c r="B11" s="6">
-        <f>IF(B4=4,78,IF(B4=2,34,56))</f>
+        <f>ROUND(IF(B4=4,78,IF(B4=2,34,56))*(B8/10),0)</f>
         <v/>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Дефолт тарифа (4 мес: 78, 2 мес: 34) или вручную</t>
+          <t>Дефолт тарифа с учетом ящиков (x1, x1.5, x2, x3) или вручную</t>
         </is>
       </c>
     </row>

</xml_diff>